<commit_message>
docs(ent-01): verificacion de Gemini, evidencia fuera de storage y conteo real
Gemini verifico ENT-01 en pantalla y dejo su bitacora sin commitear. Se sube su trabajo, se mueve la captura del recibo de storage/ a docs/06-pruebas/evidencia/ (storage/ es runtime, no repositorio) y se corrige el conteo: 315 pruebas / 1804 aserciones, porque despues de su corrida entraron las dos pruebas del Excel del padron.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/06-pruebas/PADRON-PRUEBA.xlsx
+++ b/docs/06-pruebas/PADRON-PRUEBA.xlsx
@@ -1,21 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\gestion-wings\docs\06-pruebas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0402FBC7-DDB2-4257-A0F5-5B46D98B6907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Padron" sheetId="1" r:id="rId4"/>
+    <sheet name="Padron" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Padron!$A$1:$P$1</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="152">
   <si>
     <t>DNI</t>
   </si>
@@ -423,19 +431,62 @@
   </si>
   <si>
     <t>Zárate, Clara</t>
+  </si>
+  <si>
+    <t>Periodo 7</t>
+  </si>
+  <si>
+    <t>Monto 7</t>
+  </si>
+  <si>
+    <t>Periodo 8</t>
+  </si>
+  <si>
+    <t>Monto 8</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>092026</t>
+  </si>
+  <si>
+    <t>082026</t>
+  </si>
+  <si>
+    <t>012026</t>
+  </si>
+  <si>
+    <t>072026</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>052026</t>
+  </si>
+  <si>
+    <t>062026</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>042026</t>
+  </si>
+  <si>
+    <t>032026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -462,14 +513,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="49" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -759,14 +818,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:P61"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:T61"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -815,33 +875,61 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16">
+      <c r="Q1" t="s">
+        <v>136</v>
+      </c>
+      <c r="R1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S1" t="s">
+        <v>138</v>
+      </c>
+      <c r="T1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="G2" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F2">
+        <v>52000</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H2">
+        <v>48500</v>
+      </c>
       <c r="I2" s="1"/>
       <c r="K2" s="1"/>
       <c r="M2" s="1"/>
       <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>141</v>
       </c>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -850,15 +938,18 @@
       <c r="M3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>141</v>
       </c>
       <c r="E4" s="1"/>
       <c r="G4" s="1"/>
@@ -867,15 +958,18 @@
       <c r="M4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>141</v>
       </c>
       <c r="E5" s="1"/>
       <c r="G5" s="1"/>
@@ -884,66 +978,103 @@
       <c r="M5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>115</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="1"/>
+      <c r="D6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F6">
+        <v>48500.5</v>
+      </c>
       <c r="G6" s="1"/>
       <c r="I6" s="1"/>
       <c r="K6" s="1"/>
       <c r="M6" s="1"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="1"/>
+      <c r="D7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F7">
+        <v>52000</v>
+      </c>
       <c r="G7" s="1"/>
       <c r="I7" s="1"/>
       <c r="K7" s="1"/>
       <c r="M7" s="1"/>
       <c r="O7" s="1"/>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="I8" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F8">
+        <v>48000</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H8">
+        <v>48000</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="J8">
+        <v>51000</v>
+      </c>
       <c r="K8" s="1"/>
       <c r="M8" s="1"/>
       <c r="O8" s="1"/>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>141</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="1"/>
@@ -952,15 +1083,18 @@
       <c r="M9" s="1"/>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>141</v>
       </c>
       <c r="E10" s="1"/>
       <c r="G10" s="1"/>
@@ -969,15 +1103,18 @@
       <c r="M10" s="1"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="C11" t="s">
         <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>141</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="1"/>
@@ -986,15 +1123,18 @@
       <c r="M11" s="1"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
+      </c>
+      <c r="D12" t="s">
+        <v>141</v>
       </c>
       <c r="E12" s="1"/>
       <c r="G12" s="1"/>
@@ -1003,15 +1143,18 @@
       <c r="M12" s="1"/>
       <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
         <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>141</v>
       </c>
       <c r="E13" s="1"/>
       <c r="G13" s="1"/>
@@ -1020,15 +1163,18 @@
       <c r="M13" s="1"/>
       <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D14" t="s">
+        <v>141</v>
       </c>
       <c r="E14" s="1"/>
       <c r="G14" s="1"/>
@@ -1037,15 +1183,18 @@
       <c r="M14" s="1"/>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
         <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>141</v>
       </c>
       <c r="E15" s="1"/>
       <c r="G15" s="1"/>
@@ -1054,83 +1203,123 @@
       <c r="M15" s="1"/>
       <c r="O15" s="1"/>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>127</v>
       </c>
       <c r="C16" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="D16" t="s">
+        <v>140</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F16">
+        <v>52000</v>
+      </c>
       <c r="G16" s="1"/>
       <c r="I16" s="1"/>
       <c r="K16" s="1"/>
       <c r="M16" s="1"/>
       <c r="O16" s="1"/>
     </row>
-    <row r="17" spans="1:16">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>92</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="1"/>
+      <c r="D17" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F17">
+        <v>48000</v>
+      </c>
       <c r="G17" s="1"/>
       <c r="I17" s="1"/>
       <c r="K17" s="1"/>
       <c r="M17" s="1"/>
       <c r="O17" s="1"/>
     </row>
-    <row r="18" spans="1:16">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F18">
+        <v>53000</v>
+      </c>
       <c r="G18" s="1"/>
       <c r="I18" s="1"/>
       <c r="K18" s="1"/>
       <c r="M18" s="1"/>
       <c r="O18" s="1"/>
     </row>
-    <row r="19" spans="1:16">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="G19" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="D19" t="s">
+        <v>140</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19">
+        <v>48000</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H19">
+        <v>5500.8</v>
+      </c>
       <c r="I19" s="1"/>
       <c r="K19" s="1"/>
       <c r="M19" s="1"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="1:16">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C20" t="s">
         <v>18</v>
+      </c>
+      <c r="D20" t="s">
+        <v>141</v>
       </c>
       <c r="E20" s="1"/>
       <c r="G20" s="1"/>
@@ -1139,15 +1328,18 @@
       <c r="M20" s="1"/>
       <c r="O20" s="1"/>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>134</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>135</v>
       </c>
       <c r="C21" t="s">
         <v>23</v>
+      </c>
+      <c r="D21" t="s">
+        <v>141</v>
       </c>
       <c r="E21" s="1"/>
       <c r="G21" s="1"/>
@@ -1156,32 +1348,43 @@
       <c r="M21" s="1"/>
       <c r="O21" s="1"/>
     </row>
-    <row r="22" spans="1:16">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C22" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="1"/>
+      <c r="D22" t="s">
+        <v>140</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F22">
+        <v>48000</v>
+      </c>
       <c r="G22" s="1"/>
       <c r="I22" s="1"/>
       <c r="K22" s="1"/>
       <c r="M22" s="1"/>
       <c r="O22" s="1"/>
     </row>
-    <row r="23" spans="1:16">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
         <v>18</v>
+      </c>
+      <c r="D23" t="s">
+        <v>141</v>
       </c>
       <c r="E23" s="1"/>
       <c r="G23" s="1"/>
@@ -1190,15 +1393,18 @@
       <c r="M23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
         <v>23</v>
+      </c>
+      <c r="D24" t="s">
+        <v>141</v>
       </c>
       <c r="E24" s="1"/>
       <c r="G24" s="1"/>
@@ -1207,15 +1413,18 @@
       <c r="M24" s="1"/>
       <c r="O24" s="1"/>
     </row>
-    <row r="25" spans="1:16">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>118</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>141</v>
       </c>
       <c r="E25" s="1"/>
       <c r="G25" s="1"/>
@@ -1224,15 +1433,18 @@
       <c r="M25" s="1"/>
       <c r="O25" s="1"/>
     </row>
-    <row r="26" spans="1:16">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="C26" t="s">
         <v>23</v>
+      </c>
+      <c r="D26" t="s">
+        <v>141</v>
       </c>
       <c r="E26" s="1"/>
       <c r="G26" s="1"/>
@@ -1241,7 +1453,7 @@
       <c r="M26" s="1"/>
       <c r="O26" s="1"/>
     </row>
-    <row r="27" spans="1:16">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -1250,6 +1462,9 @@
       </c>
       <c r="C27" t="s">
         <v>23</v>
+      </c>
+      <c r="D27" t="s">
+        <v>141</v>
       </c>
       <c r="E27" s="1"/>
       <c r="G27" s="1"/>
@@ -1258,15 +1473,18 @@
       <c r="M27" s="1"/>
       <c r="O27" s="1"/>
     </row>
-    <row r="28" spans="1:16">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D28" t="s">
+        <v>141</v>
       </c>
       <c r="E28" s="1"/>
       <c r="G28" s="1"/>
@@ -1275,15 +1493,18 @@
       <c r="M28" s="1"/>
       <c r="O28" s="1"/>
     </row>
-    <row r="29" spans="1:16">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>72</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="C29" t="s">
         <v>23</v>
+      </c>
+      <c r="D29" t="s">
+        <v>141</v>
       </c>
       <c r="E29" s="1"/>
       <c r="G29" s="1"/>
@@ -1292,15 +1513,18 @@
       <c r="M29" s="1"/>
       <c r="O29" s="1"/>
     </row>
-    <row r="30" spans="1:16">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="C30" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D30" t="s">
+        <v>141</v>
       </c>
       <c r="E30" s="1"/>
       <c r="G30" s="1"/>
@@ -1309,7 +1533,7 @@
       <c r="M30" s="1"/>
       <c r="O30" s="1"/>
     </row>
-    <row r="31" spans="1:16">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>76</v>
       </c>
@@ -1318,6 +1542,9 @@
       </c>
       <c r="C31" t="s">
         <v>23</v>
+      </c>
+      <c r="D31" t="s">
+        <v>141</v>
       </c>
       <c r="E31" s="1"/>
       <c r="G31" s="1"/>
@@ -1326,15 +1553,18 @@
       <c r="M31" s="1"/>
       <c r="O31" s="1"/>
     </row>
-    <row r="32" spans="1:16">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D32" t="s">
+        <v>141</v>
       </c>
       <c r="E32" s="1"/>
       <c r="G32" s="1"/>
@@ -1343,49 +1573,78 @@
       <c r="M32" s="1"/>
       <c r="O32" s="1"/>
     </row>
-    <row r="33" spans="1:16">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="B33" t="s">
-        <v>81</v>
+        <v>123</v>
       </c>
       <c r="C33" t="s">
         <v>23</v>
       </c>
-      <c r="E33" s="1"/>
+      <c r="D33" t="s">
+        <v>140</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33">
+        <v>48000</v>
+      </c>
       <c r="G33" s="1"/>
       <c r="I33" s="1"/>
       <c r="K33" s="1"/>
       <c r="M33" s="1"/>
       <c r="O33" s="1"/>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
-        <v>23</v>
-      </c>
-      <c r="E34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="I34" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="D34" t="s">
+        <v>140</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F34">
+        <v>52000</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H34">
+        <v>52000</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="J34">
+        <v>50000</v>
+      </c>
       <c r="K34" s="1"/>
       <c r="M34" s="1"/>
       <c r="O34" s="1"/>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>85</v>
+        <v>37</v>
       </c>
       <c r="C35" t="s">
         <v>23</v>
+      </c>
+      <c r="D35" t="s">
+        <v>146</v>
       </c>
       <c r="E35" s="1"/>
       <c r="G35" s="1"/>
@@ -1394,32 +1653,48 @@
       <c r="M35" s="1"/>
       <c r="O35" s="1"/>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
         <v>18</v>
       </c>
-      <c r="E36" s="1"/>
-      <c r="G36" s="1"/>
+      <c r="D36" t="s">
+        <v>140</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F36">
+        <v>52000</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H36">
+        <v>52000</v>
+      </c>
       <c r="I36" s="1"/>
       <c r="K36" s="1"/>
       <c r="M36" s="1"/>
       <c r="O36" s="1"/>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="C37" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D37" t="s">
+        <v>141</v>
       </c>
       <c r="E37" s="1"/>
       <c r="G37" s="1"/>
@@ -1428,66 +1703,93 @@
       <c r="M37" s="1"/>
       <c r="O37" s="1"/>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="B38" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="C38" t="s">
-        <v>23</v>
-      </c>
-      <c r="E38" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="D38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F38">
+        <v>51000</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
       <c r="M38" s="1"/>
       <c r="O38" s="1"/>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="C39" t="s">
-        <v>18</v>
-      </c>
-      <c r="E39" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="D39" t="s">
+        <v>140</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F39">
+        <v>52000</v>
+      </c>
       <c r="G39" s="1"/>
       <c r="I39" s="1"/>
       <c r="K39" s="1"/>
       <c r="M39" s="1"/>
       <c r="O39" s="1"/>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="C40" t="s">
         <v>23</v>
       </c>
-      <c r="E40" s="1"/>
+      <c r="D40" t="s">
+        <v>140</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F40">
+        <v>52000</v>
+      </c>
       <c r="G40" s="1"/>
       <c r="I40" s="1"/>
       <c r="K40" s="1"/>
       <c r="M40" s="1"/>
       <c r="O40" s="1"/>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="C41" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D41" t="s">
+        <v>141</v>
       </c>
       <c r="E41" s="1"/>
       <c r="G41" s="1"/>
@@ -1496,15 +1798,18 @@
       <c r="M41" s="1"/>
       <c r="O41" s="1"/>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B42" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C42" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D42" t="s">
+        <v>141</v>
       </c>
       <c r="E42" s="1"/>
       <c r="G42" s="1"/>
@@ -1513,15 +1818,18 @@
       <c r="M42" s="1"/>
       <c r="O42" s="1"/>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>98</v>
+        <v>132</v>
       </c>
       <c r="B43" t="s">
-        <v>99</v>
+        <v>133</v>
       </c>
       <c r="C43" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D43" t="s">
+        <v>141</v>
       </c>
       <c r="E43" s="1"/>
       <c r="G43" s="1"/>
@@ -1530,15 +1838,18 @@
       <c r="M43" s="1"/>
       <c r="O43" s="1"/>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B44" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="C44" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D44" t="s">
+        <v>141</v>
       </c>
       <c r="E44" s="1"/>
       <c r="G44" s="1"/>
@@ -1547,15 +1858,18 @@
       <c r="M44" s="1"/>
       <c r="O44" s="1"/>
     </row>
-    <row r="45" spans="1:16">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="C45" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D45" t="s">
+        <v>141</v>
       </c>
       <c r="E45" s="1"/>
       <c r="G45" s="1"/>
@@ -1564,15 +1878,18 @@
       <c r="M45" s="1"/>
       <c r="O45" s="1"/>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="B46" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="C46" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D46" t="s">
+        <v>141</v>
       </c>
       <c r="E46" s="1"/>
       <c r="G46" s="1"/>
@@ -1581,7 +1898,7 @@
       <c r="M46" s="1"/>
       <c r="O46" s="1"/>
     </row>
-    <row r="47" spans="1:16">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>106</v>
       </c>
@@ -1590,6 +1907,9 @@
       </c>
       <c r="C47" t="s">
         <v>23</v>
+      </c>
+      <c r="D47" t="s">
+        <v>141</v>
       </c>
       <c r="E47" s="1"/>
       <c r="G47" s="1"/>
@@ -1598,15 +1918,18 @@
       <c r="M47" s="1"/>
       <c r="O47" s="1"/>
     </row>
-    <row r="48" spans="1:16">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="B48" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D48" t="s">
+        <v>141</v>
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
@@ -1615,49 +1938,73 @@
       <c r="M48" s="1"/>
       <c r="O48" s="1"/>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="B49" t="s">
-        <v>111</v>
+        <v>71</v>
       </c>
       <c r="C49" t="s">
         <v>23</v>
       </c>
-      <c r="E49" s="1"/>
+      <c r="D49" t="s">
+        <v>140</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F49">
+        <v>48000</v>
+      </c>
       <c r="G49" s="1"/>
       <c r="I49" s="1"/>
       <c r="K49" s="1"/>
       <c r="M49" s="1"/>
       <c r="O49" s="1"/>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>112</v>
+        <v>58</v>
       </c>
       <c r="B50" t="s">
-        <v>113</v>
+        <v>59</v>
       </c>
       <c r="C50" t="s">
         <v>23</v>
       </c>
-      <c r="E50" s="1"/>
-      <c r="G50" s="1"/>
+      <c r="D50" t="s">
+        <v>140</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F50">
+        <v>48000</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H50">
+        <v>48000</v>
+      </c>
       <c r="I50" s="1"/>
       <c r="K50" s="1"/>
       <c r="M50" s="1"/>
       <c r="O50" s="1"/>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B51" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C51" t="s">
         <v>23</v>
+      </c>
+      <c r="D51" t="s">
+        <v>141</v>
       </c>
       <c r="E51" s="1"/>
       <c r="G51" s="1"/>
@@ -1666,15 +2013,18 @@
       <c r="M51" s="1"/>
       <c r="O51" s="1"/>
     </row>
-    <row r="52" spans="1:16">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="B52" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="C52" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D52" t="s">
+        <v>141</v>
       </c>
       <c r="E52" s="1"/>
       <c r="G52" s="1"/>
@@ -1683,15 +2033,18 @@
       <c r="M52" s="1"/>
       <c r="O52" s="1"/>
     </row>
-    <row r="53" spans="1:16">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="B53" t="s">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C53" t="s">
         <v>23</v>
+      </c>
+      <c r="D53" t="s">
+        <v>141</v>
       </c>
       <c r="E53" s="1"/>
       <c r="G53" s="1"/>
@@ -1700,15 +2053,18 @@
       <c r="M53" s="1"/>
       <c r="O53" s="1"/>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B54" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C54" t="s">
         <v>23</v>
+      </c>
+      <c r="D54" t="s">
+        <v>141</v>
       </c>
       <c r="E54" s="1"/>
       <c r="G54" s="1"/>
@@ -1717,15 +2073,18 @@
       <c r="M54" s="1"/>
       <c r="O54" s="1"/>
     </row>
-    <row r="55" spans="1:16">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>122</v>
+        <v>32</v>
       </c>
       <c r="B55" t="s">
-        <v>123</v>
+        <v>33</v>
       </c>
       <c r="C55" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D55" t="s">
+        <v>141</v>
       </c>
       <c r="E55" s="1"/>
       <c r="G55" s="1"/>
@@ -1734,15 +2093,18 @@
       <c r="M55" s="1"/>
       <c r="O55" s="1"/>
     </row>
-    <row r="56" spans="1:16">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>124</v>
+        <v>19</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="C56" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D56" t="s">
+        <v>141</v>
       </c>
       <c r="E56" s="1"/>
       <c r="G56" s="1"/>
@@ -1751,49 +2113,68 @@
       <c r="M56" s="1"/>
       <c r="O56" s="1"/>
     </row>
-    <row r="57" spans="1:16">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="B57" t="s">
-        <v>127</v>
+        <v>81</v>
       </c>
       <c r="C57" t="s">
         <v>23</v>
       </c>
-      <c r="E57" s="1"/>
+      <c r="D57" t="s">
+        <v>140</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F57">
+        <v>52000</v>
+      </c>
       <c r="G57" s="1"/>
       <c r="I57" s="1"/>
       <c r="K57" s="1"/>
       <c r="M57" s="1"/>
       <c r="O57" s="1"/>
     </row>
-    <row r="58" spans="1:16">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="B58" t="s">
-        <v>129</v>
+        <v>27</v>
       </c>
       <c r="C58" t="s">
         <v>23</v>
       </c>
-      <c r="E58" s="1"/>
+      <c r="D58" t="s">
+        <v>140</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F58">
+        <v>52000</v>
+      </c>
       <c r="G58" s="1"/>
       <c r="I58" s="1"/>
       <c r="K58" s="1"/>
       <c r="M58" s="1"/>
       <c r="O58" s="1"/>
     </row>
-    <row r="59" spans="1:16">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>130</v>
+        <v>54</v>
       </c>
       <c r="B59" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="C59" t="s">
         <v>18</v>
+      </c>
+      <c r="D59" t="s">
+        <v>141</v>
       </c>
       <c r="E59" s="1"/>
       <c r="G59" s="1"/>
@@ -1802,15 +2183,18 @@
       <c r="M59" s="1"/>
       <c r="O59" s="1"/>
     </row>
-    <row r="60" spans="1:16">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="B60" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="C60" t="s">
         <v>23</v>
+      </c>
+      <c r="D60" t="s">
+        <v>141</v>
       </c>
       <c r="E60" s="1"/>
       <c r="G60" s="1"/>
@@ -1819,26 +2203,74 @@
       <c r="M60" s="1"/>
       <c r="O60" s="1"/>
     </row>
-    <row r="61" spans="1:16">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>134</v>
+        <v>96</v>
       </c>
       <c r="B61" t="s">
-        <v>135</v>
+        <v>97</v>
       </c>
       <c r="C61" t="s">
-        <v>23</v>
-      </c>
-      <c r="E61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="I61" s="1"/>
-      <c r="K61" s="1"/>
-      <c r="M61" s="1"/>
-      <c r="O61" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="D61" t="s">
+        <v>140</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F61">
+        <v>50000</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H61">
+        <v>50000</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="J61">
+        <v>50000</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="L61">
+        <v>50000</v>
+      </c>
+      <c r="M61" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="N61">
+        <v>48000</v>
+      </c>
+      <c r="O61" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="P61">
+        <v>48000</v>
+      </c>
+      <c r="Q61" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="R61">
+        <v>48000</v>
+      </c>
+      <c r="S61" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="T61">
+        <v>45000</v>
+      </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <autoFilter ref="A1:P1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P61">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test(padron): montos del padron de prueba alineados a la cuota de cada alumno
Los importes cargados a mano iban de 45.000 a 52.000 y las cuotas de los planes de prueba van de 28.000 a 50.000: la deuda declarada no se parecia a lo que Wings factura. Cada mes adeudado pasa a valer la cuota del plan del alumno, con los meses de mas de tres y de mas de seis de antiguedad un 10% y un 20% mas baratos, como un aumento real. La fila 34 repetia 072026 y quedo una sola vez. Validacion aprobada: 34 deudas y 43 cierres.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/06-pruebas/PADRON-PRUEBA.xlsx
+++ b/docs/06-pruebas/PADRON-PRUEBA.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\gestion-wings\docs\06-pruebas\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0402FBC7-DDB2-4257-A0F5-5B46D98B6907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Padron" sheetId="1" r:id="rId1"/>
+    <sheet name="Padron" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Padron!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Padron'!$A$1:$P$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="152">
   <si>
     <t>DNI</t>
   </si>
@@ -73,13 +67,370 @@
     <t>Monto 6</t>
   </si>
   <si>
+    <t>Periodo 7</t>
+  </si>
+  <si>
+    <t>Monto 7</t>
+  </si>
+  <si>
+    <t>Periodo 8</t>
+  </si>
+  <si>
+    <t>Monto 8</t>
+  </si>
+  <si>
+    <t>32123456</t>
+  </si>
+  <si>
+    <t>Morales, Sofía</t>
+  </si>
+  <si>
+    <t>Patín</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>082026</t>
+  </si>
+  <si>
+    <t>092026</t>
+  </si>
+  <si>
+    <t>Fútbol</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>39281654</t>
+  </si>
+  <si>
+    <t>Godoy, Martina</t>
+  </si>
+  <si>
+    <t>39481562</t>
+  </si>
+  <si>
+    <t>Quiroga, Rocío</t>
+  </si>
+  <si>
+    <t>39562841</t>
+  </si>
+  <si>
+    <t>Serrano, Noelia</t>
+  </si>
+  <si>
+    <t>012026</t>
+  </si>
+  <si>
+    <t>39647280</t>
+  </si>
+  <si>
+    <t>Molina, Malena</t>
+  </si>
+  <si>
+    <t>39682714</t>
+  </si>
+  <si>
+    <t>Sosa, Pablo</t>
+  </si>
+  <si>
+    <t>072026</t>
+  </si>
+  <si>
+    <t>39715428</t>
+  </si>
+  <si>
+    <t>Delgado, Mariana</t>
+  </si>
+  <si>
+    <t>39724619</t>
+  </si>
+  <si>
+    <t>Giménez, Facundo</t>
+  </si>
+  <si>
+    <t>39726845</t>
+  </si>
+  <si>
+    <t>Urrutia, Ailén</t>
+  </si>
+  <si>
+    <t>39815267</t>
+  </si>
+  <si>
+    <t>Barrios, Benjamín</t>
+  </si>
+  <si>
+    <t>39862471</t>
+  </si>
+  <si>
+    <t>Cabrera, Milagros</t>
+  </si>
+  <si>
+    <t>39916473</t>
+  </si>
+  <si>
+    <t>Navarro, Kevin</t>
+  </si>
+  <si>
+    <t>39984721</t>
+  </si>
+  <si>
+    <t>Correa, Elena</t>
+  </si>
+  <si>
+    <t>40138572</t>
+  </si>
+  <si>
+    <t>Valdez, Romina</t>
+  </si>
+  <si>
+    <t>40274518</t>
+  </si>
+  <si>
+    <t>Ortega, Olivia</t>
+  </si>
+  <si>
+    <t>40291864</t>
+  </si>
+  <si>
+    <t>Pérez, Marcos</t>
+  </si>
+  <si>
+    <t>40389617</t>
+  </si>
+  <si>
+    <t>Ponce, Lorena</t>
+  </si>
+  <si>
+    <t>40468125</t>
+  </si>
+  <si>
+    <t>Díaz, Damián</t>
+  </si>
+  <si>
+    <t>40492637</t>
+  </si>
+  <si>
+    <t>Zárate, Clara</t>
+  </si>
+  <si>
+    <t>40518376</t>
+  </si>
+  <si>
+    <t>Escudero, Florencia</t>
+  </si>
+  <si>
+    <t>40537268</t>
+  </si>
+  <si>
+    <t>Luna, Iván</t>
+  </si>
+  <si>
+    <t>40615294</t>
+  </si>
+  <si>
+    <t>López, Inés</t>
+  </si>
+  <si>
+    <t>40738195</t>
+  </si>
+  <si>
+    <t>Suárez, Tatiana</t>
+  </si>
+  <si>
+    <t>40857193</t>
+  </si>
+  <si>
+    <t>Benítez, Celeste</t>
+  </si>
+  <si>
+    <t>40926713</t>
+  </si>
+  <si>
+    <t>Ibarra, Camila</t>
+  </si>
+  <si>
     <t>41627593</t>
   </si>
   <si>
     <t>Acosta, Alan</t>
   </si>
   <si>
-    <t>Fútbol</t>
+    <t>41738592</t>
+  </si>
+  <si>
+    <t>Arias, Valentina</t>
+  </si>
+  <si>
+    <t>41863957</t>
+  </si>
+  <si>
+    <t>Núñez, Natalia</t>
+  </si>
+  <si>
+    <t>41957362</t>
+  </si>
+  <si>
+    <t>Maidana, Karina</t>
+  </si>
+  <si>
+    <t>42159308</t>
+  </si>
+  <si>
+    <t>Herrera, Luciana</t>
+  </si>
+  <si>
+    <t>42370481</t>
+  </si>
+  <si>
+    <t>Toledo, Victoria</t>
+  </si>
+  <si>
+    <t>42391857</t>
+  </si>
+  <si>
+    <t>Herrera, Gonzalo</t>
+  </si>
+  <si>
+    <t>42486305</t>
+  </si>
+  <si>
+    <t>Cáceres, Eugenia</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>42509736</t>
+  </si>
+  <si>
+    <t>Cejas, Cristóbal</t>
+  </si>
+  <si>
+    <t>052026</t>
+  </si>
+  <si>
+    <t>062026</t>
+  </si>
+  <si>
+    <t>42571936</t>
+  </si>
+  <si>
+    <t>Tissera, Paola</t>
+  </si>
+  <si>
+    <t>42638195</t>
+  </si>
+  <si>
+    <t>Ramos, Nicolás</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>42691735</t>
+  </si>
+  <si>
+    <t>Domínguez, Catalina</t>
+  </si>
+  <si>
+    <t>42731596</t>
+  </si>
+  <si>
+    <t>Bustos, Daniela</t>
+  </si>
+  <si>
+    <t>42865109</t>
+  </si>
+  <si>
+    <t>Mansilla, Joaquín</t>
+  </si>
+  <si>
+    <t>42916483</t>
+  </si>
+  <si>
+    <t>Paz, Paula</t>
+  </si>
+  <si>
+    <t>43029618</t>
+  </si>
+  <si>
+    <t>Yáñez, Sofía</t>
+  </si>
+  <si>
+    <t>43057286</t>
+  </si>
+  <si>
+    <t>Vera, Ramiro</t>
+  </si>
+  <si>
+    <t>43175682</t>
+  </si>
+  <si>
+    <t>Farías, Esteban</t>
+  </si>
+  <si>
+    <t>43185072</t>
+  </si>
+  <si>
+    <t>Vargas, Bianca</t>
+  </si>
+  <si>
+    <t>43218750</t>
+  </si>
+  <si>
+    <t>Rey, Micaela</t>
+  </si>
+  <si>
+    <t>43370526</t>
+  </si>
+  <si>
+    <t>Ojeda, Lautaro</t>
+  </si>
+  <si>
+    <t>43385126</t>
+  </si>
+  <si>
+    <t>Ledesma, Josefina</t>
+  </si>
+  <si>
+    <t>43462810</t>
+  </si>
+  <si>
+    <t>Figueroa, Giselle</t>
+  </si>
+  <si>
+    <t>43529704</t>
+  </si>
+  <si>
+    <t>Roldán, Sabrina</t>
+  </si>
+  <si>
+    <t>43827019</t>
+  </si>
+  <si>
+    <t>Ferreyra, Agustina</t>
+  </si>
+  <si>
+    <t>44238951</t>
+  </si>
+  <si>
+    <t>Cuello, Renata</t>
+  </si>
+  <si>
+    <t>44672390</t>
+  </si>
+  <si>
+    <t>Rivas, Guadalupe</t>
+  </si>
+  <si>
+    <t>44760925</t>
+  </si>
+  <si>
+    <t>Cabral, Lisandro</t>
   </si>
   <si>
     <t>44851273</t>
@@ -88,19 +439,10 @@
     <t>Aguirre, Bautista</t>
   </si>
   <si>
-    <t>41738592</t>
-  </si>
-  <si>
-    <t>Arias, Valentina</t>
-  </si>
-  <si>
-    <t>Patín</t>
-  </si>
-  <si>
-    <t>39815267</t>
-  </si>
-  <si>
-    <t>Barrios, Benjamín</t>
+    <t>44917264</t>
+  </si>
+  <si>
+    <t>Medina, Julieta</t>
   </si>
   <si>
     <t>45012387</t>
@@ -109,208 +451,16 @@
     <t>Benegas, Abril</t>
   </si>
   <si>
-    <t>40857193</t>
-  </si>
-  <si>
-    <t>Benítez, Celeste</t>
-  </si>
-  <si>
-    <t>42731596</t>
-  </si>
-  <si>
-    <t>Bustos, Daniela</t>
-  </si>
-  <si>
-    <t>44760925</t>
-  </si>
-  <si>
-    <t>Cabral, Lisandro</t>
-  </si>
-  <si>
-    <t>39862471</t>
-  </si>
-  <si>
-    <t>Cabrera, Milagros</t>
-  </si>
-  <si>
-    <t>42486305</t>
-  </si>
-  <si>
-    <t>Cáceres, Eugenia</t>
-  </si>
-  <si>
-    <t>42509736</t>
-  </si>
-  <si>
-    <t>Cejas, Cristóbal</t>
-  </si>
-  <si>
-    <t>39984721</t>
-  </si>
-  <si>
-    <t>Correa, Elena</t>
-  </si>
-  <si>
-    <t>44238951</t>
-  </si>
-  <si>
-    <t>Cuello, Renata</t>
-  </si>
-  <si>
-    <t>39715428</t>
-  </si>
-  <si>
-    <t>Delgado, Mariana</t>
-  </si>
-  <si>
-    <t>40468125</t>
-  </si>
-  <si>
-    <t>Díaz, Damián</t>
-  </si>
-  <si>
-    <t>42691735</t>
-  </si>
-  <si>
-    <t>Domínguez, Catalina</t>
-  </si>
-  <si>
-    <t>40518376</t>
-  </si>
-  <si>
-    <t>Escudero, Florencia</t>
-  </si>
-  <si>
-    <t>43175682</t>
-  </si>
-  <si>
-    <t>Farías, Esteban</t>
-  </si>
-  <si>
     <t>45094618</t>
   </si>
   <si>
     <t>Ferrari, Valentino</t>
   </si>
   <si>
-    <t>43827019</t>
-  </si>
-  <si>
-    <t>Ferreyra, Agustina</t>
-  </si>
-  <si>
-    <t>43462810</t>
-  </si>
-  <si>
-    <t>Figueroa, Giselle</t>
-  </si>
-  <si>
-    <t>39724619</t>
-  </si>
-  <si>
-    <t>Giménez, Facundo</t>
-  </si>
-  <si>
-    <t>39281654</t>
-  </si>
-  <si>
-    <t>Godoy, Martina</t>
-  </si>
-  <si>
-    <t>42391857</t>
-  </si>
-  <si>
-    <t>Herrera, Gonzalo</t>
-  </si>
-  <si>
-    <t>42159308</t>
-  </si>
-  <si>
-    <t>Herrera, Luciana</t>
-  </si>
-  <si>
-    <t>40926713</t>
-  </si>
-  <si>
-    <t>Ibarra, Camila</t>
-  </si>
-  <si>
-    <t>43385126</t>
-  </si>
-  <si>
-    <t>Ledesma, Josefina</t>
-  </si>
-  <si>
-    <t>40615294</t>
-  </si>
-  <si>
-    <t>López, Inés</t>
-  </si>
-  <si>
-    <t>40537268</t>
-  </si>
-  <si>
-    <t>Luna, Iván</t>
-  </si>
-  <si>
-    <t>41957362</t>
-  </si>
-  <si>
-    <t>Maidana, Karina</t>
-  </si>
-  <si>
-    <t>42865109</t>
-  </si>
-  <si>
-    <t>Mansilla, Joaquín</t>
-  </si>
-  <si>
-    <t>44917264</t>
-  </si>
-  <si>
-    <t>Medina, Julieta</t>
-  </si>
-  <si>
-    <t>39647280</t>
-  </si>
-  <si>
-    <t>Molina, Malena</t>
-  </si>
-  <si>
-    <t>32123456</t>
-  </si>
-  <si>
-    <t>Morales, Sofía</t>
-  </si>
-  <si>
-    <t>39916473</t>
-  </si>
-  <si>
-    <t>Navarro, Kevin</t>
-  </si>
-  <si>
-    <t>41863957</t>
-  </si>
-  <si>
-    <t>Núñez, Natalia</t>
-  </si>
-  <si>
-    <t>43370526</t>
-  </si>
-  <si>
-    <t>Ojeda, Lautaro</t>
-  </si>
-  <si>
-    <t>40274518</t>
-  </si>
-  <si>
-    <t>Ortega, Olivia</t>
-  </si>
-  <si>
-    <t>42916483</t>
-  </si>
-  <si>
-    <t>Paz, Paula</t>
+    <t>45183726</t>
+  </si>
+  <si>
+    <t>Sandoval, Emilia</t>
   </si>
   <si>
     <t>45329018</t>
@@ -319,174 +469,23 @@
     <t>Peralta, Thiago</t>
   </si>
   <si>
-    <t>40291864</t>
-  </si>
-  <si>
-    <t>Pérez, Marcos</t>
-  </si>
-  <si>
-    <t>40389617</t>
-  </si>
-  <si>
-    <t>Ponce, Lorena</t>
-  </si>
-  <si>
-    <t>39481562</t>
-  </si>
-  <si>
-    <t>Quiroga, Rocío</t>
-  </si>
-  <si>
-    <t>42638195</t>
-  </si>
-  <si>
-    <t>Ramos, Nicolás</t>
-  </si>
-  <si>
-    <t>43218750</t>
-  </si>
-  <si>
-    <t>Rey, Micaela</t>
-  </si>
-  <si>
-    <t>44672390</t>
-  </si>
-  <si>
-    <t>Rivas, Guadalupe</t>
-  </si>
-  <si>
-    <t>43529704</t>
-  </si>
-  <si>
-    <t>Roldán, Sabrina</t>
-  </si>
-  <si>
-    <t>45183726</t>
-  </si>
-  <si>
-    <t>Sandoval, Emilia</t>
-  </si>
-  <si>
-    <t>39562841</t>
-  </si>
-  <si>
-    <t>Serrano, Noelia</t>
-  </si>
-  <si>
-    <t>39682714</t>
-  </si>
-  <si>
-    <t>Sosa, Pablo</t>
-  </si>
-  <si>
-    <t>40738195</t>
-  </si>
-  <si>
-    <t>Suárez, Tatiana</t>
-  </si>
-  <si>
-    <t>42571936</t>
-  </si>
-  <si>
-    <t>Tissera, Paola</t>
-  </si>
-  <si>
-    <t>42370481</t>
-  </si>
-  <si>
-    <t>Toledo, Victoria</t>
-  </si>
-  <si>
-    <t>39726845</t>
-  </si>
-  <si>
-    <t>Urrutia, Ailén</t>
-  </si>
-  <si>
-    <t>40138572</t>
-  </si>
-  <si>
-    <t>Valdez, Romina</t>
-  </si>
-  <si>
-    <t>43185072</t>
-  </si>
-  <si>
-    <t>Vargas, Bianca</t>
-  </si>
-  <si>
-    <t>43057286</t>
-  </si>
-  <si>
-    <t>Vera, Ramiro</t>
-  </si>
-  <si>
-    <t>43029618</t>
-  </si>
-  <si>
-    <t>Yáñez, Sofía</t>
-  </si>
-  <si>
-    <t>40492637</t>
-  </si>
-  <si>
-    <t>Zárate, Clara</t>
-  </si>
-  <si>
-    <t>Periodo 7</t>
-  </si>
-  <si>
-    <t>Monto 7</t>
-  </si>
-  <si>
-    <t>Periodo 8</t>
-  </si>
-  <si>
-    <t>Monto 8</t>
-  </si>
-  <si>
-    <t>si</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>092026</t>
-  </si>
-  <si>
-    <t>082026</t>
-  </si>
-  <si>
-    <t>012026</t>
-  </si>
-  <si>
-    <t>072026</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>052026</t>
-  </si>
-  <si>
-    <t>062026</t>
-  </si>
-  <si>
-    <t>SI</t>
+    <t>032026</t>
   </si>
   <si>
     <t>042026</t>
-  </si>
-  <si>
-    <t>032026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -513,22 +512,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="49" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -818,15 +809,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:T61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="9.140625" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" customWidth="true" style="0"/>
+    <col min="2" max="2" width="19.140625" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -876,60 +870,60 @@
         <v>15</v>
       </c>
       <c r="Q1" t="s">
-        <v>136</v>
+        <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>137</v>
+        <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>138</v>
+        <v>18</v>
       </c>
       <c r="T1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
-        <v>140</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="F2">
-        <v>52000</v>
+        <v>30000.0</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>143</v>
+        <v>25</v>
       </c>
       <c r="H2">
-        <v>48500</v>
+        <v>30000.0</v>
       </c>
       <c r="I2" s="1"/>
       <c r="K2" s="1"/>
       <c r="M2" s="1"/>
       <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -938,18 +932,18 @@
       <c r="M3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E4" s="1"/>
       <c r="G4" s="1"/>
@@ -958,18 +952,18 @@
       <c r="M4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1"/>
       <c r="G5" s="1"/>
@@ -978,24 +972,24 @@
       <c r="M5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
-        <v>140</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>144</v>
+        <v>34</v>
       </c>
       <c r="F6">
-        <v>48500.5</v>
+        <v>40000.0</v>
       </c>
       <c r="G6" s="1"/>
       <c r="I6" s="1"/>
@@ -1003,24 +997,24 @@
       <c r="M6" s="1"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
         <v>23</v>
       </c>
-      <c r="D7" t="s">
-        <v>140</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F7">
-        <v>52000</v>
+        <v>43000.0</v>
       </c>
       <c r="G7" s="1"/>
       <c r="I7" s="1"/>
@@ -1028,53 +1022,53 @@
       <c r="M7" s="1"/>
       <c r="O7" s="1"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>140</v>
+        <v>23</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>143</v>
+        <v>39</v>
       </c>
       <c r="F8">
-        <v>48000</v>
+        <v>48000.0</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>145</v>
+        <v>24</v>
       </c>
       <c r="H8">
-        <v>48000</v>
+        <v>48000.0</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="J8">
-        <v>51000</v>
+        <v>48000.0</v>
       </c>
       <c r="K8" s="1"/>
       <c r="M8" s="1"/>
       <c r="O8" s="1"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="1"/>
@@ -1083,18 +1077,18 @@
       <c r="M9" s="1"/>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1"/>
       <c r="G10" s="1"/>
@@ -1103,18 +1097,18 @@
       <c r="M10" s="1"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>124</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>125</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="1"/>
@@ -1123,18 +1117,18 @@
       <c r="M11" s="1"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E12" s="1"/>
       <c r="G12" s="1"/>
@@ -1143,18 +1137,18 @@
       <c r="M12" s="1"/>
       <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E13" s="1"/>
       <c r="G13" s="1"/>
@@ -1163,18 +1157,18 @@
       <c r="M13" s="1"/>
       <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E14" s="1"/>
       <c r="G14" s="1"/>
@@ -1183,18 +1177,18 @@
       <c r="M14" s="1"/>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E15" s="1"/>
       <c r="G15" s="1"/>
@@ -1203,24 +1197,24 @@
       <c r="M15" s="1"/>
       <c r="O15" s="1"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>126</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
-        <v>127</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
         <v>23</v>
       </c>
-      <c r="D16" t="s">
-        <v>140</v>
-      </c>
       <c r="E16" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F16">
-        <v>52000</v>
+        <v>43000.0</v>
       </c>
       <c r="G16" s="1"/>
       <c r="I16" s="1"/>
@@ -1228,24 +1222,24 @@
       <c r="M16" s="1"/>
       <c r="O16" s="1"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" t="s">
         <v>23</v>
       </c>
-      <c r="D17" t="s">
-        <v>140</v>
-      </c>
       <c r="E17" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F17">
-        <v>48000</v>
+        <v>50000.0</v>
       </c>
       <c r="G17" s="1"/>
       <c r="I17" s="1"/>
@@ -1253,24 +1247,24 @@
       <c r="M17" s="1"/>
       <c r="O17" s="1"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
-        <v>140</v>
+        <v>23</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F18">
-        <v>53000</v>
+        <v>48000.0</v>
       </c>
       <c r="G18" s="1"/>
       <c r="I18" s="1"/>
@@ -1278,48 +1272,48 @@
       <c r="M18" s="1"/>
       <c r="O18" s="1"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="C19" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" t="s">
         <v>23</v>
       </c>
-      <c r="D19" t="s">
-        <v>140</v>
-      </c>
       <c r="E19" s="1" t="s">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="F19">
-        <v>48000</v>
+        <v>43000.0</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>143</v>
+        <v>25</v>
       </c>
       <c r="H19">
-        <v>5500.8</v>
+        <v>43000.0</v>
       </c>
       <c r="I19" s="1"/>
       <c r="K19" s="1"/>
       <c r="M19" s="1"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D20" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E20" s="1"/>
       <c r="G20" s="1"/>
@@ -1328,18 +1322,18 @@
       <c r="M20" s="1"/>
       <c r="O20" s="1"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20">
       <c r="A21" t="s">
-        <v>134</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>135</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D21" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E21" s="1"/>
       <c r="G21" s="1"/>
@@ -1348,24 +1342,24 @@
       <c r="M21" s="1"/>
       <c r="O21" s="1"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C22" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" t="s">
         <v>23</v>
       </c>
-      <c r="D22" t="s">
-        <v>140</v>
-      </c>
       <c r="E22" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F22">
-        <v>48000</v>
+        <v>50000.0</v>
       </c>
       <c r="G22" s="1"/>
       <c r="I22" s="1"/>
@@ -1373,18 +1367,18 @@
       <c r="M22" s="1"/>
       <c r="O22" s="1"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20">
       <c r="A23" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E23" s="1"/>
       <c r="G23" s="1"/>
@@ -1393,18 +1387,18 @@
       <c r="M23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20">
       <c r="A24" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E24" s="1"/>
       <c r="G24" s="1"/>
@@ -1413,18 +1407,18 @@
       <c r="M24" s="1"/>
       <c r="O24" s="1"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20">
       <c r="A25" t="s">
-        <v>118</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="C25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E25" s="1"/>
       <c r="G25" s="1"/>
@@ -1433,18 +1427,18 @@
       <c r="M25" s="1"/>
       <c r="O25" s="1"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E26" s="1"/>
       <c r="G26" s="1"/>
@@ -1453,18 +1447,18 @@
       <c r="M26" s="1"/>
       <c r="O26" s="1"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E27" s="1"/>
       <c r="G27" s="1"/>
@@ -1473,18 +1467,18 @@
       <c r="M27" s="1"/>
       <c r="O27" s="1"/>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>79</v>
       </c>
       <c r="C28" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D28" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E28" s="1"/>
       <c r="G28" s="1"/>
@@ -1493,18 +1487,18 @@
       <c r="M28" s="1"/>
       <c r="O28" s="1"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20">
       <c r="A29" t="s">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E29" s="1"/>
       <c r="G29" s="1"/>
@@ -1513,18 +1507,18 @@
       <c r="M29" s="1"/>
       <c r="O29" s="1"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20">
       <c r="A30" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E30" s="1"/>
       <c r="G30" s="1"/>
@@ -1533,18 +1527,18 @@
       <c r="M30" s="1"/>
       <c r="O30" s="1"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E31" s="1"/>
       <c r="G31" s="1"/>
@@ -1553,18 +1547,18 @@
       <c r="M31" s="1"/>
       <c r="O31" s="1"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="B32" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E32" s="1"/>
       <c r="G32" s="1"/>
@@ -1573,24 +1567,24 @@
       <c r="M32" s="1"/>
       <c r="O32" s="1"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>88</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" t="s">
         <v>23</v>
       </c>
-      <c r="D33" t="s">
-        <v>140</v>
-      </c>
       <c r="E33" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F33">
-        <v>48000</v>
+        <v>30000.0</v>
       </c>
       <c r="G33" s="1"/>
       <c r="I33" s="1"/>
@@ -1598,53 +1592,48 @@
       <c r="M33" s="1"/>
       <c r="O33" s="1"/>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20">
       <c r="A34" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D34" t="s">
-        <v>140</v>
+        <v>23</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="F34">
-        <v>52000</v>
+        <v>28000.0</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>143</v>
+        <v>24</v>
       </c>
       <c r="H34">
-        <v>52000</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J34">
-        <v>50000</v>
-      </c>
+        <v>28000.0</v>
+      </c>
+      <c r="I34" s="1"/>
       <c r="K34" s="1"/>
       <c r="M34" s="1"/>
       <c r="O34" s="1"/>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="C35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>146</v>
+        <v>94</v>
       </c>
       <c r="E35" s="1"/>
       <c r="G35" s="1"/>
@@ -1653,48 +1642,48 @@
       <c r="M35" s="1"/>
       <c r="O35" s="1"/>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>95</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D36" t="s">
-        <v>140</v>
+        <v>23</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>147</v>
+        <v>97</v>
       </c>
       <c r="F36">
-        <v>52000</v>
+        <v>25000.0</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>148</v>
+        <v>98</v>
       </c>
       <c r="H36">
-        <v>52000</v>
+        <v>25000.0</v>
       </c>
       <c r="I36" s="1"/>
       <c r="K36" s="1"/>
       <c r="M36" s="1"/>
       <c r="O36" s="1"/>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20">
       <c r="A37" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="B37" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="C37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E37" s="1"/>
       <c r="G37" s="1"/>
@@ -1703,24 +1692,24 @@
       <c r="M37" s="1"/>
       <c r="O37" s="1"/>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20">
       <c r="A38" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C38" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D38" t="s">
-        <v>149</v>
+        <v>103</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F38">
-        <v>51000</v>
+        <v>28000.0</v>
       </c>
       <c r="G38" s="1"/>
       <c r="I38" s="1"/>
@@ -1728,24 +1717,24 @@
       <c r="M38" s="1"/>
       <c r="O38" s="1"/>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20">
       <c r="A39" t="s">
-        <v>48</v>
+        <v>104</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>105</v>
       </c>
       <c r="C39" t="s">
+        <v>22</v>
+      </c>
+      <c r="D39" t="s">
         <v>23</v>
       </c>
-      <c r="D39" t="s">
-        <v>140</v>
-      </c>
       <c r="E39" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F39">
-        <v>52000</v>
+        <v>35000.0</v>
       </c>
       <c r="G39" s="1"/>
       <c r="I39" s="1"/>
@@ -1753,24 +1742,24 @@
       <c r="M39" s="1"/>
       <c r="O39" s="1"/>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20">
       <c r="A40" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="B40" t="s">
-        <v>31</v>
+        <v>107</v>
       </c>
       <c r="C40" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" t="s">
         <v>23</v>
       </c>
-      <c r="D40" t="s">
-        <v>140</v>
-      </c>
       <c r="E40" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F40">
-        <v>52000</v>
+        <v>30000.0</v>
       </c>
       <c r="G40" s="1"/>
       <c r="I40" s="1"/>
@@ -1778,18 +1767,18 @@
       <c r="M40" s="1"/>
       <c r="O40" s="1"/>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>108</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="C41" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D41" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E41" s="1"/>
       <c r="G41" s="1"/>
@@ -1798,18 +1787,18 @@
       <c r="M41" s="1"/>
       <c r="O41" s="1"/>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20">
       <c r="A42" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="B42" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="C42" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E42" s="1"/>
       <c r="G42" s="1"/>
@@ -1818,18 +1807,18 @@
       <c r="M42" s="1"/>
       <c r="O42" s="1"/>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20">
       <c r="A43" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="B43" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="C43" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E43" s="1"/>
       <c r="G43" s="1"/>
@@ -1838,18 +1827,18 @@
       <c r="M43" s="1"/>
       <c r="O43" s="1"/>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20">
       <c r="A44" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="B44" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="C44" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D44" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E44" s="1"/>
       <c r="G44" s="1"/>
@@ -1858,18 +1847,18 @@
       <c r="M44" s="1"/>
       <c r="O44" s="1"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>116</v>
       </c>
       <c r="B45" t="s">
-        <v>53</v>
+        <v>117</v>
       </c>
       <c r="C45" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D45" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E45" s="1"/>
       <c r="G45" s="1"/>
@@ -1878,18 +1867,18 @@
       <c r="M45" s="1"/>
       <c r="O45" s="1"/>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20">
       <c r="A46" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B46" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C46" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E46" s="1"/>
       <c r="G46" s="1"/>
@@ -1898,18 +1887,18 @@
       <c r="M46" s="1"/>
       <c r="O46" s="1"/>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20">
       <c r="A47" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="B47" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="C47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E47" s="1"/>
       <c r="G47" s="1"/>
@@ -1918,18 +1907,18 @@
       <c r="M47" s="1"/>
       <c r="O47" s="1"/>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20">
       <c r="A48" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>123</v>
       </c>
       <c r="C48" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D48" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
@@ -1938,24 +1927,24 @@
       <c r="M48" s="1"/>
       <c r="O48" s="1"/>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20">
       <c r="A49" t="s">
-        <v>70</v>
+        <v>124</v>
       </c>
       <c r="B49" t="s">
-        <v>71</v>
+        <v>125</v>
       </c>
       <c r="C49" t="s">
+        <v>22</v>
+      </c>
+      <c r="D49" t="s">
         <v>23</v>
       </c>
-      <c r="D49" t="s">
-        <v>140</v>
-      </c>
       <c r="E49" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F49">
-        <v>48000</v>
+        <v>30000.0</v>
       </c>
       <c r="G49" s="1"/>
       <c r="I49" s="1"/>
@@ -1963,48 +1952,48 @@
       <c r="M49" s="1"/>
       <c r="O49" s="1"/>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20">
       <c r="A50" t="s">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="B50" t="s">
-        <v>59</v>
+        <v>127</v>
       </c>
       <c r="C50" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" t="s">
         <v>23</v>
       </c>
-      <c r="D50" t="s">
-        <v>140</v>
-      </c>
       <c r="E50" s="1" t="s">
-        <v>142</v>
+        <v>24</v>
       </c>
       <c r="F50">
-        <v>48000</v>
+        <v>35000.0</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>143</v>
+        <v>25</v>
       </c>
       <c r="H50">
-        <v>48000</v>
+        <v>35000.0</v>
       </c>
       <c r="I50" s="1"/>
       <c r="K50" s="1"/>
       <c r="M50" s="1"/>
       <c r="O50" s="1"/>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20">
       <c r="A51" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="B51" t="s">
-        <v>111</v>
+        <v>129</v>
       </c>
       <c r="C51" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E51" s="1"/>
       <c r="G51" s="1"/>
@@ -2013,18 +2002,18 @@
       <c r="M51" s="1"/>
       <c r="O51" s="1"/>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20">
       <c r="A52" t="s">
-        <v>56</v>
+        <v>130</v>
       </c>
       <c r="B52" t="s">
-        <v>57</v>
+        <v>131</v>
       </c>
       <c r="C52" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E52" s="1"/>
       <c r="G52" s="1"/>
@@ -2033,18 +2022,18 @@
       <c r="M52" s="1"/>
       <c r="O52" s="1"/>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20">
       <c r="A53" t="s">
-        <v>42</v>
+        <v>132</v>
       </c>
       <c r="B53" t="s">
-        <v>43</v>
+        <v>133</v>
       </c>
       <c r="C53" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E53" s="1"/>
       <c r="G53" s="1"/>
@@ -2053,18 +2042,18 @@
       <c r="M53" s="1"/>
       <c r="O53" s="1"/>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20">
       <c r="A54" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="B54" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="C54" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E54" s="1"/>
       <c r="G54" s="1"/>
@@ -2073,18 +2062,18 @@
       <c r="M54" s="1"/>
       <c r="O54" s="1"/>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20">
       <c r="A55" t="s">
-        <v>32</v>
+        <v>136</v>
       </c>
       <c r="B55" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
       <c r="C55" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D55" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E55" s="1"/>
       <c r="G55" s="1"/>
@@ -2093,18 +2082,18 @@
       <c r="M55" s="1"/>
       <c r="O55" s="1"/>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20">
       <c r="A56" t="s">
-        <v>19</v>
+        <v>138</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
+        <v>139</v>
       </c>
       <c r="C56" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D56" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E56" s="1"/>
       <c r="G56" s="1"/>
@@ -2113,24 +2102,24 @@
       <c r="M56" s="1"/>
       <c r="O56" s="1"/>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20">
       <c r="A57" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="B57" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="C57" t="s">
+        <v>22</v>
+      </c>
+      <c r="D57" t="s">
         <v>23</v>
       </c>
-      <c r="D57" t="s">
-        <v>140</v>
-      </c>
       <c r="E57" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F57">
-        <v>52000</v>
+        <v>50000.0</v>
       </c>
       <c r="G57" s="1"/>
       <c r="I57" s="1"/>
@@ -2138,24 +2127,24 @@
       <c r="M57" s="1"/>
       <c r="O57" s="1"/>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20">
       <c r="A58" t="s">
-        <v>26</v>
+        <v>142</v>
       </c>
       <c r="B58" t="s">
-        <v>27</v>
+        <v>143</v>
       </c>
       <c r="C58" t="s">
+        <v>22</v>
+      </c>
+      <c r="D58" t="s">
         <v>23</v>
       </c>
-      <c r="D58" t="s">
-        <v>140</v>
-      </c>
       <c r="E58" s="1" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="F58">
-        <v>52000</v>
+        <v>43000.0</v>
       </c>
       <c r="G58" s="1"/>
       <c r="I58" s="1"/>
@@ -2163,18 +2152,18 @@
       <c r="M58" s="1"/>
       <c r="O58" s="1"/>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20">
       <c r="A59" t="s">
-        <v>54</v>
+        <v>144</v>
       </c>
       <c r="B59" t="s">
-        <v>55</v>
+        <v>145</v>
       </c>
       <c r="C59" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D59" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E59" s="1"/>
       <c r="G59" s="1"/>
@@ -2183,18 +2172,18 @@
       <c r="M59" s="1"/>
       <c r="O59" s="1"/>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20">
       <c r="A60" t="s">
-        <v>112</v>
+        <v>146</v>
       </c>
       <c r="B60" t="s">
-        <v>113</v>
+        <v>147</v>
       </c>
       <c r="C60" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D60" t="s">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="E60" s="1"/>
       <c r="G60" s="1"/>
@@ -2203,74 +2192,72 @@
       <c r="M60" s="1"/>
       <c r="O60" s="1"/>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20">
       <c r="A61" t="s">
-        <v>96</v>
+        <v>148</v>
       </c>
       <c r="B61" t="s">
+        <v>149</v>
+      </c>
+      <c r="C61" t="s">
+        <v>26</v>
+      </c>
+      <c r="D61" t="s">
+        <v>23</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F61">
+        <v>30500.0</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H61">
+        <v>30500.0</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="J61">
+        <v>34000.0</v>
+      </c>
+      <c r="K61" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C61" t="s">
-        <v>18</v>
-      </c>
-      <c r="D61" t="s">
-        <v>140</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F61">
-        <v>50000</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="H61">
-        <v>50000</v>
-      </c>
-      <c r="I61" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J61">
-        <v>50000</v>
-      </c>
-      <c r="K61" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="L61">
-        <v>50000</v>
+        <v>34000.0</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="N61">
-        <v>48000</v>
+        <v>34000.0</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>150</v>
+        <v>39</v>
       </c>
       <c r="P61">
-        <v>48000</v>
+        <v>38000.0</v>
       </c>
       <c r="Q61" s="1" t="s">
-        <v>151</v>
+        <v>24</v>
       </c>
       <c r="R61">
-        <v>48000</v>
+        <v>38000.0</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>144</v>
+        <v>25</v>
       </c>
       <c r="T61">
-        <v>45000</v>
+        <v>38000.0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P61">
-      <sortCondition ref="A1"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:P1"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>